<commit_message>
added c++ cstdint headers explicit int cast when reading time of connection
</commit_message>
<xml_diff>
--- a/tests/formats/mfn_excel/MFN_example.xlsx
+++ b/tests/formats/mfn_excel/MFN_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\en986\Documents\Projects\Alltours\generalized_agv_path_finding\tests\formats\mfn_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{852381D4-135C-4AF6-B76A-E90E0C0D8691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83D4E26-2946-4B58-955F-71C16BA193B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="228" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
+    <workbookView xWindow="30612" yWindow="228" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{B8DE84FF-B3E8-4D87-8A95-BDBF8C6662ED}"/>
   </bookViews>
   <sheets>
     <sheet name="NetworkNodes" sheetId="3" r:id="rId1"/>
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -184,6 +184,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,7 +708,7 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="6">
         <v>90</v>
       </c>
       <c r="E2" t="s">

</xml_diff>